<commit_message>
Add public contact findings to lead list
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CExgX3LnZkdy4AwdW7vCVh
</commit_message>
<xml_diff>
--- a/leads/GrassCrafts_Leads_Diwali_2026.xlsx
+++ b/leads/GrassCrafts_Leads_Diwali_2026.xlsx
@@ -644,7 +644,11 @@
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr"/>
-      <c r="H2" s="5" t="inlineStr"/>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>Email not found; HQ Mumbai</t>
+        </is>
+      </c>
       <c r="I2" s="4" t="inlineStr">
         <is>
           <t>Not contacted</t>
@@ -804,7 +808,11 @@
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr"/>
-      <c r="H6" s="5" t="inlineStr"/>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>hello@aukerajewellery.com (general) / contact@aukerajewellery.com (support) – from third-party listing indiacustomercare.com, verify on aukerajewellery.com; ph 90354 54656</t>
+        </is>
+      </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
           <t>Not contacted</t>
@@ -1084,7 +1092,11 @@
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr"/>
-      <c r="H13" s="5" t="inlineStr"/>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t>Email not public; website offineeds.com</t>
+        </is>
+      </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
           <t>Not contacted</t>
@@ -1124,7 +1136,11 @@
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr"/>
-      <c r="H14" s="5" t="inlineStr"/>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>Ph +91 80 4456 6931 (IndiaMART); website thegivingtree.in; proprietor Leena Munot</t>
+        </is>
+      </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
           <t>Not contacted</t>
@@ -1684,7 +1700,11 @@
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr"/>
-      <c r="H28" s="5" t="inlineStr"/>
+      <c r="H28" s="5" t="inlineStr">
+        <is>
+          <t>Actually Goa-based (founder Nafisa Afonso Sheikh); contact via WedMeGood/WeddingSutra profile</t>
+        </is>
+      </c>
       <c r="I28" s="4" t="inlineStr">
         <is>
           <t>Not contacted</t>
@@ -2420,7 +2440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:H24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2430,6 +2450,7 @@
     <col width="22" customWidth="1" min="5" max="5"/>
     <col width="50" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2468,6 +2489,11 @@
           <t>Reorder pitch sent?</t>
         </is>
       </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Public contact found (verify)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
@@ -2487,6 +2513,11 @@
       <c r="E2" s="5" t="inlineStr"/>
       <c r="F2" s="5" t="inlineStr"/>
       <c r="G2" s="5" t="inlineStr"/>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Restaurant 'Van Lavino', Nallagandla, Hyderabad; partners Abhijeet Pai, Harish Ramnani; no public email</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="n">
@@ -2510,6 +2541,11 @@
       <c r="E3" s="5" t="inlineStr"/>
       <c r="F3" s="5" t="inlineStr"/>
       <c r="G3" s="5" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>HCL/Shiv Nadar Foundation, A-9 Sec 3 Noida, ph +91 120 3667000</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
@@ -2533,6 +2569,11 @@
       <c r="E4" s="5" t="inlineStr"/>
       <c r="F4" s="5" t="inlineStr"/>
       <c r="G4" s="5" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Brand: Birdy's (NSE SME: BIRDYS), birdys.in; ph +91 22 5002 9517; only public email is ipo@birdys.in (investor use – not for sales)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
@@ -2575,6 +2616,11 @@
       <c r="E6" s="5" t="inlineStr"/>
       <c r="F6" s="5" t="inlineStr"/>
       <c r="G6" s="5" t="inlineStr"/>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Founder &amp; CEO: Pankaj Dutta (RocketReach); no public email</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
@@ -2636,6 +2682,11 @@
       <c r="E9" s="5" t="inlineStr"/>
       <c r="F9" s="5" t="inlineStr"/>
       <c r="G9" s="5" t="inlineStr"/>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Website vbev.co.in; ph +91 22 4250 5130 (Datanyze, unverified)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
@@ -2750,6 +2801,11 @@
       <c r="E15" s="5" t="inlineStr"/>
       <c r="F15" s="5" t="inlineStr"/>
       <c r="G15" s="5" t="inlineStr"/>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Founder Priyanka Singh; no public email</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
@@ -2788,6 +2844,11 @@
       <c r="E17" s="5" t="inlineStr"/>
       <c r="F17" s="5" t="inlineStr"/>
       <c r="G17" s="5" t="inlineStr"/>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Likely 'Kevasiya', West Punjabi Bagh, New Delhi – IndiaMART, contact Divya Sethi, ph +91 80 4573 2944</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
@@ -2925,6 +2986,11 @@
       <c r="E24" s="5" t="inlineStr"/>
       <c r="F24" s="5" t="inlineStr"/>
       <c r="G24" s="5" t="inlineStr"/>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>No public listing found</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:G24"/>

</xml_diff>

<commit_message>
Expand lead list to 96 prospects across 6 segments
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CExgX3LnZkdy4AwdW7vCVh
</commit_message>
<xml_diff>
--- a/leads/GrassCrafts_Leads_Diwali_2026.xlsx
+++ b/leads/GrassCrafts_Leads_Diwali_2026.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Existing Clients" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Prospects'!$A$1:$L$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Prospects'!$A$1:$L$95</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'LinkedIn Searches'!$A$1:$E$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Existing Clients'!$A$1:$G$24</definedName>
   </definedNames>
@@ -539,7 +539,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L41"/>
+  <dimension ref="A1:L95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2238,10 +2238,2170 @@
         </is>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" s="4" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>Diamond jewellery (gift boxes)</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>Tanishq (Titan)</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>Bengaluru / pan-India</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="inlineStr"/>
+      <c r="F42" s="4" t="inlineStr">
+        <is>
+          <t>Branded handwoven Kauna/Sabai jewellery boxes &amp; trays as premium, plastic-free packaging</t>
+        </is>
+      </c>
+      <c r="G42" s="5" t="inlineStr"/>
+      <c r="H42" s="5" t="inlineStr"/>
+      <c r="I42" s="4" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J42" s="5" t="inlineStr"/>
+      <c r="K42" s="5" t="inlineStr"/>
+      <c r="L42" s="4" t="inlineStr">
+        <is>
+          <t>https://www.giva.co/blogs/tales/top-10-certified-lab-grown-diamond-jewellery-brands-in-india-2026-guide</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>Diamond jewellery (gift boxes)</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>Ivana Jewels</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>Surat</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="inlineStr"/>
+      <c r="F43" s="4" t="inlineStr">
+        <is>
+          <t>Branded handwoven Kauna/Sabai jewellery boxes &amp; trays as premium, plastic-free packaging</t>
+        </is>
+      </c>
+      <c r="G43" s="5" t="inlineStr"/>
+      <c r="H43" s="5" t="inlineStr"/>
+      <c r="I43" s="4" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J43" s="5" t="inlineStr"/>
+      <c r="K43" s="5" t="inlineStr"/>
+      <c r="L43" s="4" t="inlineStr">
+        <is>
+          <t>https://earthlyjewels.co/blogs/blog/lab-grown-diamond-jewellery-brands-in-india</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>Diamond jewellery (gift boxes)</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>Kapu Gems</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>Surat</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="inlineStr"/>
+      <c r="F44" s="4" t="inlineStr">
+        <is>
+          <t>Gift boxes for their B2B/retail jewellery clients</t>
+        </is>
+      </c>
+      <c r="G44" s="5" t="inlineStr"/>
+      <c r="H44" s="5" t="inlineStr"/>
+      <c r="I44" s="4" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J44" s="5" t="inlineStr"/>
+      <c r="K44" s="5" t="inlineStr"/>
+      <c r="L44" s="4" t="inlineStr">
+        <is>
+          <t>https://raremonds.com/best-natural-diamond-suppliers-in-india/</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>Diamond jewellery (gift boxes)</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t>Zahra Diamonds</t>
+        </is>
+      </c>
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>Surat</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr"/>
+      <c r="F45" s="4" t="inlineStr">
+        <is>
+          <t>Gift boxes for their B2B/retail jewellery clients</t>
+        </is>
+      </c>
+      <c r="G45" s="5" t="inlineStr"/>
+      <c r="H45" s="5" t="inlineStr"/>
+      <c r="I45" s="4" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J45" s="5" t="inlineStr"/>
+      <c r="K45" s="5" t="inlineStr"/>
+      <c r="L45" s="4" t="inlineStr">
+        <is>
+          <t>https://raremonds.com/best-natural-diamond-suppliers-in-india/</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>Diamond jewellery (gift boxes)</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>Samkit Ratna</t>
+        </is>
+      </c>
+      <c r="D46" s="4" t="inlineStr">
+        <is>
+          <t>Mumbai</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr"/>
+      <c r="F46" s="4" t="inlineStr">
+        <is>
+          <t>Gift boxes for their B2B/retail jewellery clients</t>
+        </is>
+      </c>
+      <c r="G46" s="5" t="inlineStr"/>
+      <c r="H46" s="5" t="inlineStr"/>
+      <c r="I46" s="4" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J46" s="5" t="inlineStr"/>
+      <c r="K46" s="5" t="inlineStr"/>
+      <c r="L46" s="4" t="inlineStr">
+        <is>
+          <t>https://raremonds.com/best-natural-diamond-suppliers-in-india/</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>Diamond jewellery (gift boxes)</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>Nvision Diamjewel LLP</t>
+        </is>
+      </c>
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>Mumbai</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="inlineStr"/>
+      <c r="F47" s="4" t="inlineStr">
+        <is>
+          <t>Gift boxes for their B2B/retail jewellery clients</t>
+        </is>
+      </c>
+      <c r="G47" s="5" t="inlineStr"/>
+      <c r="H47" s="5" t="inlineStr"/>
+      <c r="I47" s="4" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J47" s="5" t="inlineStr"/>
+      <c r="K47" s="5" t="inlineStr"/>
+      <c r="L47" s="4" t="inlineStr">
+        <is>
+          <t>https://raremonds.com/best-natural-diamond-suppliers-in-india/</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="4" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>Diamond jewellery (gift boxes)</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>Hari Krishna Exports (Kisna brand)</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t>Surat / Mumbai</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr"/>
+      <c r="F48" s="4" t="inlineStr">
+        <is>
+          <t>Branded handwoven Kauna/Sabai jewellery boxes &amp; trays as premium, plastic-free packaging</t>
+        </is>
+      </c>
+      <c r="G48" s="5" t="inlineStr"/>
+      <c r="H48" s="5" t="inlineStr"/>
+      <c r="I48" s="4" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J48" s="5" t="inlineStr"/>
+      <c r="K48" s="5" t="inlineStr"/>
+      <c r="L48" s="4" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Hari_Krishna_Exports</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>Diamond jewellery (gift boxes)</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="inlineStr">
+        <is>
+          <t>Kiran Gems</t>
+        </is>
+      </c>
+      <c r="D49" s="4" t="inlineStr">
+        <is>
+          <t>Surat</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="inlineStr"/>
+      <c r="F49" s="4" t="inlineStr">
+        <is>
+          <t>Corporate/festive gifting for employees &amp; trade partners</t>
+        </is>
+      </c>
+      <c r="G49" s="5" t="inlineStr"/>
+      <c r="H49" s="5" t="inlineStr"/>
+      <c r="I49" s="4" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J49" s="5" t="inlineStr"/>
+      <c r="K49" s="5" t="inlineStr"/>
+      <c r="L49" s="4" t="inlineStr">
+        <is>
+          <t>https://en.wikipedia.org/wiki/Kiran_Gems</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="4" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t>Corporate gifting companies</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="inlineStr">
+        <is>
+          <t>Kari by Kriti</t>
+        </is>
+      </c>
+      <c r="D50" s="4" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr"/>
+      <c r="F50" s="4" t="inlineStr">
+        <is>
+          <t>Artisan-made gifting partner – co-branded handwoven hampers</t>
+        </is>
+      </c>
+      <c r="G50" s="5" t="inlineStr"/>
+      <c r="H50" s="5" t="inlineStr"/>
+      <c r="I50" s="4" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J50" s="5" t="inlineStr"/>
+      <c r="K50" s="5" t="inlineStr"/>
+      <c r="L50" s="4" t="inlineStr">
+        <is>
+          <t>https://www.karibykriti.com/blogs/news/sustainable-corporate-diwali-gifts-india-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>Corporate gifting companies</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="inlineStr">
+        <is>
+          <t>The Good Road</t>
+        </is>
+      </c>
+      <c r="D51" s="4" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="inlineStr"/>
+      <c r="F51" s="4" t="inlineStr">
+        <is>
+          <t>Add handwoven grass products to their sustainable gift range</t>
+        </is>
+      </c>
+      <c r="G51" s="5" t="inlineStr"/>
+      <c r="H51" s="5" t="inlineStr"/>
+      <c r="I51" s="4" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J51" s="5" t="inlineStr"/>
+      <c r="K51" s="5" t="inlineStr"/>
+      <c r="L51" s="4" t="inlineStr">
+        <is>
+          <t>https://www.thegoodroad.in/blogs/all-blogs/8-sustainable-diwali-gift-ideas-for-employees-that-they-ll-actually-use-in-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t>Corporate gifting companies</t>
+        </is>
+      </c>
+      <c r="C52" s="4" t="inlineStr">
+        <is>
+          <t>Box N Bond</t>
+        </is>
+      </c>
+      <c r="D52" s="4" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr"/>
+      <c r="F52" s="4" t="inlineStr">
+        <is>
+          <t>White-label handwoven hampers, trays and desk sets they can resell</t>
+        </is>
+      </c>
+      <c r="G52" s="5" t="inlineStr"/>
+      <c r="H52" s="5" t="inlineStr"/>
+      <c r="I52" s="4" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J52" s="5" t="inlineStr"/>
+      <c r="K52" s="5" t="inlineStr"/>
+      <c r="L52" s="4" t="inlineStr">
+        <is>
+          <t>https://boxnbond.com/eco-friendly-corporate-gifts-india/</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" s="4" t="inlineStr">
+        <is>
+          <t>Corporate gifting companies</t>
+        </is>
+      </c>
+      <c r="C53" s="4" t="inlineStr">
+        <is>
+          <t>IGP Corporate (eco collection)</t>
+        </is>
+      </c>
+      <c r="D53" s="4" t="inlineStr">
+        <is>
+          <t>Mumbai</t>
+        </is>
+      </c>
+      <c r="E53" s="5" t="inlineStr"/>
+      <c r="F53" s="4" t="inlineStr">
+        <is>
+          <t>White-label handwoven hampers, trays and desk sets they can resell</t>
+        </is>
+      </c>
+      <c r="G53" s="5" t="inlineStr"/>
+      <c r="H53" s="5" t="inlineStr"/>
+      <c r="I53" s="4" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J53" s="5" t="inlineStr"/>
+      <c r="K53" s="5" t="inlineStr"/>
+      <c r="L53" s="4" t="inlineStr">
+        <is>
+          <t>https://www.igp.com/corporate-gifts/ecofriendly-collections</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" s="4" t="inlineStr">
+        <is>
+          <t>Corporate gifting companies</t>
+        </is>
+      </c>
+      <c r="C54" s="4" t="inlineStr">
+        <is>
+          <t>Zaggle (gifting)</t>
+        </is>
+      </c>
+      <c r="D54" s="4" t="inlineStr">
+        <is>
+          <t>Hyderabad</t>
+        </is>
+      </c>
+      <c r="E54" s="5" t="inlineStr"/>
+      <c r="F54" s="4" t="inlineStr">
+        <is>
+          <t>White-label handwoven hampers, trays and desk sets they can resell</t>
+        </is>
+      </c>
+      <c r="G54" s="5" t="inlineStr"/>
+      <c r="H54" s="5" t="inlineStr"/>
+      <c r="I54" s="4" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J54" s="5" t="inlineStr"/>
+      <c r="K54" s="5" t="inlineStr"/>
+      <c r="L54" s="4" t="inlineStr">
+        <is>
+          <t>https://www.zaggle.in/knowledge-hub/blog/top-10-corporate-diwali-gifting-trends-indian-companies-are-following-in-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="4" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" s="4" t="inlineStr">
+        <is>
+          <t>Corporate gifting companies</t>
+        </is>
+      </c>
+      <c r="C55" s="4" t="inlineStr">
+        <is>
+          <t>Regal Corporate Gift</t>
+        </is>
+      </c>
+      <c r="D55" s="4" t="inlineStr">
+        <is>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="E55" s="5" t="inlineStr"/>
+      <c r="F55" s="4" t="inlineStr">
+        <is>
+          <t>White-label handwoven hampers, trays and desk sets they can resell</t>
+        </is>
+      </c>
+      <c r="G55" s="5" t="inlineStr"/>
+      <c r="H55" s="5" t="inlineStr"/>
+      <c r="I55" s="4" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J55" s="5" t="inlineStr"/>
+      <c r="K55" s="5" t="inlineStr"/>
+      <c r="L55" s="4" t="inlineStr">
+        <is>
+          <t>https://regalcorporategift.com/shop/happilo-dry-fruit-gift-hamper-tulip-as-corporate-gifts/</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" s="4" t="inlineStr">
+        <is>
+          <t>Wedding &amp; event planners</t>
+        </is>
+      </c>
+      <c r="C56" s="4" t="inlineStr">
+        <is>
+          <t>Opus Kreation</t>
+        </is>
+      </c>
+      <c r="D56" s="4" t="inlineStr">
+        <is>
+          <t>Kolkata</t>
+        </is>
+      </c>
+      <c r="E56" s="5" t="inlineStr"/>
+      <c r="F56" s="4" t="inlineStr">
+        <is>
+          <t>Wedding return-gift &amp; trousseau hampers (Haldi/Mehendi/Godh Bharai) in bulk</t>
+        </is>
+      </c>
+      <c r="G56" s="5" t="inlineStr"/>
+      <c r="H56" s="5" t="inlineStr"/>
+      <c r="I56" s="4" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J56" s="5" t="inlineStr"/>
+      <c r="K56" s="5" t="inlineStr"/>
+      <c r="L56" s="4" t="inlineStr">
+        <is>
+          <t>https://lbb.in/kolkata/wedding-planners-kolkata/</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" s="4" t="inlineStr">
+        <is>
+          <t>Wedding &amp; event planners</t>
+        </is>
+      </c>
+      <c r="C57" s="4" t="inlineStr">
+        <is>
+          <t>Veydaa</t>
+        </is>
+      </c>
+      <c r="D57" s="4" t="inlineStr">
+        <is>
+          <t>Kolkata</t>
+        </is>
+      </c>
+      <c r="E57" s="5" t="inlineStr"/>
+      <c r="F57" s="4" t="inlineStr">
+        <is>
+          <t>Wedding return-gift &amp; trousseau hampers (Haldi/Mehendi/Godh Bharai) in bulk</t>
+        </is>
+      </c>
+      <c r="G57" s="5" t="inlineStr"/>
+      <c r="H57" s="5" t="inlineStr"/>
+      <c r="I57" s="4" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J57" s="5" t="inlineStr"/>
+      <c r="K57" s="5" t="inlineStr"/>
+      <c r="L57" s="4" t="inlineStr">
+        <is>
+          <t>https://lbb.in/kolkata/wedding-planners-kolkata/</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" s="4" t="inlineStr">
+        <is>
+          <t>Wedding &amp; event planners</t>
+        </is>
+      </c>
+      <c r="C58" s="4" t="inlineStr">
+        <is>
+          <t>The Paisley Project</t>
+        </is>
+      </c>
+      <c r="D58" s="4" t="inlineStr">
+        <is>
+          <t>Kolkata / Bengaluru</t>
+        </is>
+      </c>
+      <c r="E58" s="5" t="inlineStr"/>
+      <c r="F58" s="4" t="inlineStr">
+        <is>
+          <t>Wedding return-gift &amp; trousseau hampers (Haldi/Mehendi/Godh Bharai) in bulk</t>
+        </is>
+      </c>
+      <c r="G58" s="5" t="inlineStr"/>
+      <c r="H58" s="5" t="inlineStr"/>
+      <c r="I58" s="4" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J58" s="5" t="inlineStr"/>
+      <c r="K58" s="5" t="inlineStr"/>
+      <c r="L58" s="4" t="inlineStr">
+        <is>
+          <t>https://weddingsutra.com/wedding-vendors/wedding-planners/</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="4" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" s="4" t="inlineStr">
+        <is>
+          <t>Wedding &amp; event planners</t>
+        </is>
+      </c>
+      <c r="C59" s="4" t="inlineStr">
+        <is>
+          <t>Dhaaga Events</t>
+        </is>
+      </c>
+      <c r="D59" s="4" t="inlineStr">
+        <is>
+          <t>Kolkata</t>
+        </is>
+      </c>
+      <c r="E59" s="5" t="inlineStr"/>
+      <c r="F59" s="4" t="inlineStr">
+        <is>
+          <t>Wedding return-gift &amp; trousseau hampers (Haldi/Mehendi/Godh Bharai) in bulk</t>
+        </is>
+      </c>
+      <c r="G59" s="5" t="inlineStr"/>
+      <c r="H59" s="5" t="inlineStr"/>
+      <c r="I59" s="4" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J59" s="5" t="inlineStr"/>
+      <c r="K59" s="5" t="inlineStr"/>
+      <c r="L59" s="4" t="inlineStr">
+        <is>
+          <t>https://weddingsutra.com/wedding-vendors/wedding-planners/</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" s="4" t="inlineStr">
+        <is>
+          <t>Wedding &amp; event planners</t>
+        </is>
+      </c>
+      <c r="C60" s="4" t="inlineStr">
+        <is>
+          <t>Panigrahana Weddings</t>
+        </is>
+      </c>
+      <c r="D60" s="4" t="inlineStr">
+        <is>
+          <t>Bengaluru / Goa / Coorg</t>
+        </is>
+      </c>
+      <c r="E60" s="5" t="inlineStr"/>
+      <c r="F60" s="4" t="inlineStr">
+        <is>
+          <t>Wedding return-gift &amp; trousseau hampers (Haldi/Mehendi/Godh Bharai) in bulk</t>
+        </is>
+      </c>
+      <c r="G60" s="5" t="inlineStr"/>
+      <c r="H60" s="5" t="inlineStr"/>
+      <c r="I60" s="4" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J60" s="5" t="inlineStr"/>
+      <c r="K60" s="5" t="inlineStr"/>
+      <c r="L60" s="4" t="inlineStr">
+        <is>
+          <t>https://panigrahana.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" s="4" t="inlineStr">
+        <is>
+          <t>Wedding &amp; event planners</t>
+        </is>
+      </c>
+      <c r="C61" s="4" t="inlineStr">
+        <is>
+          <t>Abhinava Weddings</t>
+        </is>
+      </c>
+      <c r="D61" s="4" t="inlineStr">
+        <is>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="E61" s="5" t="inlineStr"/>
+      <c r="F61" s="4" t="inlineStr">
+        <is>
+          <t>Wedding return-gift &amp; trousseau hampers (Haldi/Mehendi/Godh Bharai) in bulk</t>
+        </is>
+      </c>
+      <c r="G61" s="5" t="inlineStr"/>
+      <c r="H61" s="5" t="inlineStr"/>
+      <c r="I61" s="4" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J61" s="5" t="inlineStr"/>
+      <c r="K61" s="5" t="inlineStr"/>
+      <c r="L61" s="4" t="inlineStr">
+        <is>
+          <t>https://www.bookmywed.in/blog/best-destination-wedding-planners-in-bangalore-for-a-picture-perfect-celebration</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="4" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" s="4" t="inlineStr">
+        <is>
+          <t>Wedding &amp; event planners</t>
+        </is>
+      </c>
+      <c r="C62" s="4" t="inlineStr">
+        <is>
+          <t>AIRA Wedding Planners</t>
+        </is>
+      </c>
+      <c r="D62" s="4" t="inlineStr">
+        <is>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="E62" s="5" t="inlineStr"/>
+      <c r="F62" s="4" t="inlineStr">
+        <is>
+          <t>Wedding return-gift &amp; trousseau hampers (Haldi/Mehendi/Godh Bharai) in bulk</t>
+        </is>
+      </c>
+      <c r="G62" s="5" t="inlineStr"/>
+      <c r="H62" s="5" t="inlineStr"/>
+      <c r="I62" s="4" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J62" s="5" t="inlineStr"/>
+      <c r="K62" s="5" t="inlineStr"/>
+      <c r="L62" s="4" t="inlineStr">
+        <is>
+          <t>https://www.bookmywed.in/blog/best-destination-wedding-planners-in-bangalore-for-a-picture-perfect-celebration</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="4" t="n">
+        <v>62</v>
+      </c>
+      <c r="B63" s="4" t="inlineStr">
+        <is>
+          <t>Wedding &amp; event planners</t>
+        </is>
+      </c>
+      <c r="C63" s="4" t="inlineStr">
+        <is>
+          <t>Best Day Ever by Deepika Shetty</t>
+        </is>
+      </c>
+      <c r="D63" s="4" t="inlineStr">
+        <is>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="E63" s="5" t="inlineStr"/>
+      <c r="F63" s="4" t="inlineStr">
+        <is>
+          <t>Wedding return-gift &amp; trousseau hampers (Haldi/Mehendi/Godh Bharai) in bulk</t>
+        </is>
+      </c>
+      <c r="G63" s="5" t="inlineStr"/>
+      <c r="H63" s="5" t="inlineStr"/>
+      <c r="I63" s="4" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J63" s="5" t="inlineStr"/>
+      <c r="K63" s="5" t="inlineStr"/>
+      <c r="L63" s="4" t="inlineStr">
+        <is>
+          <t>https://www.bookmywed.in/blog/best-destination-wedding-planners-in-bangalore-for-a-picture-perfect-celebration</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="4" t="n">
+        <v>63</v>
+      </c>
+      <c r="B64" s="4" t="inlineStr">
+        <is>
+          <t>Wedding &amp; event planners</t>
+        </is>
+      </c>
+      <c r="C64" s="4" t="inlineStr">
+        <is>
+          <t>Bling It On</t>
+        </is>
+      </c>
+      <c r="D64" s="4" t="inlineStr">
+        <is>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="E64" s="5" t="inlineStr"/>
+      <c r="F64" s="4" t="inlineStr">
+        <is>
+          <t>Wedding return-gift &amp; trousseau hampers (Haldi/Mehendi/Godh Bharai) in bulk</t>
+        </is>
+      </c>
+      <c r="G64" s="5" t="inlineStr"/>
+      <c r="H64" s="5" t="inlineStr"/>
+      <c r="I64" s="4" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J64" s="5" t="inlineStr"/>
+      <c r="K64" s="5" t="inlineStr"/>
+      <c r="L64" s="4" t="inlineStr">
+        <is>
+          <t>https://www.bookmywed.in/blog/best-destination-wedding-planners-in-bangalore-for-a-picture-perfect-celebration</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="4" t="n">
+        <v>64</v>
+      </c>
+      <c r="B65" s="4" t="inlineStr">
+        <is>
+          <t>Wedding &amp; event planners</t>
+        </is>
+      </c>
+      <c r="C65" s="4" t="inlineStr">
+        <is>
+          <t>G-Unit Events</t>
+        </is>
+      </c>
+      <c r="D65" s="4" t="inlineStr">
+        <is>
+          <t>Bengaluru / Goa</t>
+        </is>
+      </c>
+      <c r="E65" s="5" t="inlineStr"/>
+      <c r="F65" s="4" t="inlineStr">
+        <is>
+          <t>Wedding return-gift &amp; trousseau hampers (Haldi/Mehendi/Godh Bharai) in bulk</t>
+        </is>
+      </c>
+      <c r="G65" s="5" t="inlineStr"/>
+      <c r="H65" s="5" t="inlineStr"/>
+      <c r="I65" s="4" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J65" s="5" t="inlineStr"/>
+      <c r="K65" s="5" t="inlineStr"/>
+      <c r="L65" s="4" t="inlineStr">
+        <is>
+          <t>https://www.gunitevents.com/destination-wedding-planner-Bangalore.php</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="4" t="n">
+        <v>65</v>
+      </c>
+      <c r="B66" s="4" t="inlineStr">
+        <is>
+          <t>Wedding &amp; event planners</t>
+        </is>
+      </c>
+      <c r="C66" s="4" t="inlineStr">
+        <is>
+          <t>Rings &amp; Roses</t>
+        </is>
+      </c>
+      <c r="D66" s="4" t="inlineStr">
+        <is>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="E66" s="5" t="inlineStr"/>
+      <c r="F66" s="4" t="inlineStr">
+        <is>
+          <t>Wedding return-gift &amp; trousseau hampers (Haldi/Mehendi/Godh Bharai) in bulk</t>
+        </is>
+      </c>
+      <c r="G66" s="5" t="inlineStr"/>
+      <c r="H66" s="5" t="inlineStr"/>
+      <c r="I66" s="4" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J66" s="5" t="inlineStr"/>
+      <c r="K66" s="5" t="inlineStr"/>
+      <c r="L66" s="4" t="inlineStr">
+        <is>
+          <t>https://shaandaarevents.com/top-10-destination-wedding-planners-in-india/</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="4" t="n">
+        <v>66</v>
+      </c>
+      <c r="B67" s="4" t="inlineStr">
+        <is>
+          <t>Wedding &amp; event planners</t>
+        </is>
+      </c>
+      <c r="C67" s="4" t="inlineStr">
+        <is>
+          <t>FNP Weddings (Ferns N Petals)</t>
+        </is>
+      </c>
+      <c r="D67" s="4" t="inlineStr">
+        <is>
+          <t>Goa / Bengaluru / Delhi</t>
+        </is>
+      </c>
+      <c r="E67" s="5" t="inlineStr"/>
+      <c r="F67" s="4" t="inlineStr">
+        <is>
+          <t>Wedding return-gift &amp; trousseau hampers (Haldi/Mehendi/Godh Bharai) in bulk</t>
+        </is>
+      </c>
+      <c r="G67" s="5" t="inlineStr"/>
+      <c r="H67" s="5" t="inlineStr"/>
+      <c r="I67" s="4" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J67" s="5" t="inlineStr"/>
+      <c r="K67" s="5" t="inlineStr"/>
+      <c r="L67" s="4" t="inlineStr">
+        <is>
+          <t>https://panigrahana.com/best-destination-wedding-planners-india-2026.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="4" t="n">
+        <v>67</v>
+      </c>
+      <c r="B68" s="4" t="inlineStr">
+        <is>
+          <t>Wedding &amp; event planners</t>
+        </is>
+      </c>
+      <c r="C68" s="4" t="inlineStr">
+        <is>
+          <t>Wedlock Weddings by Vima</t>
+        </is>
+      </c>
+      <c r="D68" s="4" t="inlineStr">
+        <is>
+          <t>Bengaluru / Goa</t>
+        </is>
+      </c>
+      <c r="E68" s="5" t="inlineStr"/>
+      <c r="F68" s="4" t="inlineStr">
+        <is>
+          <t>Wedding return-gift &amp; trousseau hampers (Haldi/Mehendi/Godh Bharai) in bulk</t>
+        </is>
+      </c>
+      <c r="G68" s="5" t="inlineStr"/>
+      <c r="H68" s="5" t="inlineStr"/>
+      <c r="I68" s="4" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J68" s="5" t="inlineStr"/>
+      <c r="K68" s="5" t="inlineStr"/>
+      <c r="L68" s="4" t="inlineStr">
+        <is>
+          <t>https://panigrahana.com/best-destination-wedding-planners-india-2026.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="4" t="n">
+        <v>68</v>
+      </c>
+      <c r="B69" s="4" t="inlineStr">
+        <is>
+          <t>Wedding &amp; event planners</t>
+        </is>
+      </c>
+      <c r="C69" s="4" t="inlineStr">
+        <is>
+          <t>Exotic Goa Events</t>
+        </is>
+      </c>
+      <c r="D69" s="4" t="inlineStr">
+        <is>
+          <t>Goa</t>
+        </is>
+      </c>
+      <c r="E69" s="5" t="inlineStr"/>
+      <c r="F69" s="4" t="inlineStr">
+        <is>
+          <t>Wedding return-gift &amp; trousseau hampers (Haldi/Mehendi/Godh Bharai) in bulk</t>
+        </is>
+      </c>
+      <c r="G69" s="5" t="inlineStr"/>
+      <c r="H69" s="5" t="inlineStr"/>
+      <c r="I69" s="4" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J69" s="5" t="inlineStr"/>
+      <c r="K69" s="5" t="inlineStr"/>
+      <c r="L69" s="4" t="inlineStr">
+        <is>
+          <t>https://panigrahana.com/best-destination-wedding-planners-india-2026.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="4" t="n">
+        <v>69</v>
+      </c>
+      <c r="B70" s="4" t="inlineStr">
+        <is>
+          <t>Trousseau / wedding gift packers</t>
+        </is>
+      </c>
+      <c r="C70" s="4" t="inlineStr">
+        <is>
+          <t>Grace The Packing Studio</t>
+        </is>
+      </c>
+      <c r="D70" s="4" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="E70" s="5" t="inlineStr"/>
+      <c r="F70" s="4" t="inlineStr">
+        <is>
+          <t>Supply handwoven trays, baskets and boxes as bases for their trousseau &amp; gift packing</t>
+        </is>
+      </c>
+      <c r="G70" s="5" t="inlineStr"/>
+      <c r="H70" s="5" t="inlineStr"/>
+      <c r="I70" s="4" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J70" s="5" t="inlineStr"/>
+      <c r="K70" s="5" t="inlineStr"/>
+      <c r="L70" s="4" t="inlineStr">
+        <is>
+          <t>https://www.gracethepackingstudio.com/</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="4" t="n">
+        <v>70</v>
+      </c>
+      <c r="B71" s="4" t="inlineStr">
+        <is>
+          <t>Trousseau / wedding gift packers</t>
+        </is>
+      </c>
+      <c r="C71" s="4" t="inlineStr">
+        <is>
+          <t>Trouzzaano</t>
+        </is>
+      </c>
+      <c r="D71" s="4" t="inlineStr">
+        <is>
+          <t>Delhi (Wazirpur)</t>
+        </is>
+      </c>
+      <c r="E71" s="5" t="inlineStr"/>
+      <c r="F71" s="4" t="inlineStr">
+        <is>
+          <t>Supply handwoven trays, baskets and boxes as bases for their trousseau &amp; gift packing</t>
+        </is>
+      </c>
+      <c r="G71" s="5" t="inlineStr"/>
+      <c r="H71" s="5" t="inlineStr"/>
+      <c r="I71" s="4" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J71" s="5" t="inlineStr"/>
+      <c r="K71" s="5" t="inlineStr"/>
+      <c r="L71" s="4" t="inlineStr">
+        <is>
+          <t>https://www.weddingwire.in/trousseau-packing</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="4" t="n">
+        <v>71</v>
+      </c>
+      <c r="B72" s="4" t="inlineStr">
+        <is>
+          <t>Trousseau / wedding gift packers</t>
+        </is>
+      </c>
+      <c r="C72" s="4" t="inlineStr">
+        <is>
+          <t>Anytime Gift Packing</t>
+        </is>
+      </c>
+      <c r="D72" s="4" t="inlineStr">
+        <is>
+          <t>Delhi (Rohini)</t>
+        </is>
+      </c>
+      <c r="E72" s="5" t="inlineStr"/>
+      <c r="F72" s="4" t="inlineStr">
+        <is>
+          <t>Supply handwoven trays, baskets and boxes as bases for their trousseau &amp; gift packing</t>
+        </is>
+      </c>
+      <c r="G72" s="5" t="inlineStr"/>
+      <c r="H72" s="5" t="inlineStr"/>
+      <c r="I72" s="4" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J72" s="5" t="inlineStr"/>
+      <c r="K72" s="5" t="inlineStr"/>
+      <c r="L72" s="4" t="inlineStr">
+        <is>
+          <t>https://www.weddingwire.in/trousseau-packing</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="B73" s="4" t="inlineStr">
+        <is>
+          <t>Trousseau / wedding gift packers</t>
+        </is>
+      </c>
+      <c r="C73" s="4" t="inlineStr">
+        <is>
+          <t>R Square Designs</t>
+        </is>
+      </c>
+      <c r="D73" s="4" t="inlineStr">
+        <is>
+          <t>Delhi NCR</t>
+        </is>
+      </c>
+      <c r="E73" s="5" t="inlineStr"/>
+      <c r="F73" s="4" t="inlineStr">
+        <is>
+          <t>Supply handwoven trays, baskets and boxes as bases for their trousseau &amp; gift packing</t>
+        </is>
+      </c>
+      <c r="G73" s="5" t="inlineStr"/>
+      <c r="H73" s="5" t="inlineStr"/>
+      <c r="I73" s="4" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J73" s="5" t="inlineStr"/>
+      <c r="K73" s="5" t="inlineStr"/>
+      <c r="L73" s="4" t="inlineStr">
+        <is>
+          <t>https://www.wedmegood.com/vendors/all/trousseau-packers/</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="4" t="n">
+        <v>73</v>
+      </c>
+      <c r="B74" s="4" t="inlineStr">
+        <is>
+          <t>Trousseau / wedding gift packers</t>
+        </is>
+      </c>
+      <c r="C74" s="4" t="inlineStr">
+        <is>
+          <t>Splendor by Simmi Pahwa</t>
+        </is>
+      </c>
+      <c r="D74" s="4" t="inlineStr">
+        <is>
+          <t>Delhi NCR</t>
+        </is>
+      </c>
+      <c r="E74" s="5" t="inlineStr"/>
+      <c r="F74" s="4" t="inlineStr">
+        <is>
+          <t>Supply handwoven trays, baskets and boxes as bases for their trousseau &amp; gift packing</t>
+        </is>
+      </c>
+      <c r="G74" s="5" t="inlineStr"/>
+      <c r="H74" s="5" t="inlineStr"/>
+      <c r="I74" s="4" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J74" s="5" t="inlineStr"/>
+      <c r="K74" s="5" t="inlineStr"/>
+      <c r="L74" s="4" t="inlineStr">
+        <is>
+          <t>https://www.wedmegood.com/vendors/all/trousseau-packers/</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="4" t="n">
+        <v>74</v>
+      </c>
+      <c r="B75" s="4" t="inlineStr">
+        <is>
+          <t>Trousseau / wedding gift packers</t>
+        </is>
+      </c>
+      <c r="C75" s="4" t="inlineStr">
+        <is>
+          <t>Wrap It Up by Chahat</t>
+        </is>
+      </c>
+      <c r="D75" s="4" t="inlineStr">
+        <is>
+          <t>Delhi NCR</t>
+        </is>
+      </c>
+      <c r="E75" s="5" t="inlineStr"/>
+      <c r="F75" s="4" t="inlineStr">
+        <is>
+          <t>Supply handwoven trays, baskets and boxes as bases for their trousseau &amp; gift packing</t>
+        </is>
+      </c>
+      <c r="G75" s="5" t="inlineStr"/>
+      <c r="H75" s="5" t="inlineStr"/>
+      <c r="I75" s="4" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J75" s="5" t="inlineStr"/>
+      <c r="K75" s="5" t="inlineStr"/>
+      <c r="L75" s="4" t="inlineStr">
+        <is>
+          <t>https://www.wedmegood.com/vendors/all/trousseau-packers/</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="4" t="n">
+        <v>75</v>
+      </c>
+      <c r="B76" s="4" t="inlineStr">
+        <is>
+          <t>Trousseau / wedding gift packers</t>
+        </is>
+      </c>
+      <c r="C76" s="4" t="inlineStr">
+        <is>
+          <t>Kanhai Creations</t>
+        </is>
+      </c>
+      <c r="D76" s="4" t="inlineStr">
+        <is>
+          <t>Mumbai (Borivali)</t>
+        </is>
+      </c>
+      <c r="E76" s="5" t="inlineStr"/>
+      <c r="F76" s="4" t="inlineStr">
+        <is>
+          <t>Supply handwoven trays, baskets and boxes as bases for their trousseau &amp; gift packing</t>
+        </is>
+      </c>
+      <c r="G76" s="5" t="inlineStr"/>
+      <c r="H76" s="5" t="inlineStr"/>
+      <c r="I76" s="4" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J76" s="5" t="inlineStr"/>
+      <c r="K76" s="5" t="inlineStr"/>
+      <c r="L76" s="4" t="inlineStr">
+        <is>
+          <t>https://www.wedmegood.com/vendors/mumbai/trousseau-packers/</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="4" t="n">
+        <v>76</v>
+      </c>
+      <c r="B77" s="4" t="inlineStr">
+        <is>
+          <t>Trousseau / wedding gift packers</t>
+        </is>
+      </c>
+      <c r="C77" s="4" t="inlineStr">
+        <is>
+          <t>Love and Hamper</t>
+        </is>
+      </c>
+      <c r="D77" s="4" t="inlineStr">
+        <is>
+          <t>Mumbai</t>
+        </is>
+      </c>
+      <c r="E77" s="5" t="inlineStr"/>
+      <c r="F77" s="4" t="inlineStr">
+        <is>
+          <t>Supply handwoven trays, baskets and boxes as bases for their trousseau &amp; gift packing</t>
+        </is>
+      </c>
+      <c r="G77" s="5" t="inlineStr"/>
+      <c r="H77" s="5" t="inlineStr"/>
+      <c r="I77" s="4" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J77" s="5" t="inlineStr"/>
+      <c r="K77" s="5" t="inlineStr"/>
+      <c r="L77" s="4" t="inlineStr">
+        <is>
+          <t>https://www.wedmegood.com/vendors/mumbai/trousseau-packers/</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="4" t="n">
+        <v>77</v>
+      </c>
+      <c r="B78" s="4" t="inlineStr">
+        <is>
+          <t>Trousseau / wedding gift packers</t>
+        </is>
+      </c>
+      <c r="C78" s="4" t="inlineStr">
+        <is>
+          <t>Wrap N Joy</t>
+        </is>
+      </c>
+      <c r="D78" s="4" t="inlineStr">
+        <is>
+          <t>Mumbai</t>
+        </is>
+      </c>
+      <c r="E78" s="5" t="inlineStr"/>
+      <c r="F78" s="4" t="inlineStr">
+        <is>
+          <t>Supply handwoven trays, baskets and boxes as bases for their trousseau &amp; gift packing</t>
+        </is>
+      </c>
+      <c r="G78" s="5" t="inlineStr"/>
+      <c r="H78" s="5" t="inlineStr"/>
+      <c r="I78" s="4" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J78" s="5" t="inlineStr"/>
+      <c r="K78" s="5" t="inlineStr"/>
+      <c r="L78" s="4" t="inlineStr">
+        <is>
+          <t>https://www.wedmegood.com/vendors/mumbai/trousseau-packers/</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="4" t="n">
+        <v>78</v>
+      </c>
+      <c r="B79" s="4" t="inlineStr">
+        <is>
+          <t>Trousseau / wedding gift packers</t>
+        </is>
+      </c>
+      <c r="C79" s="4" t="inlineStr">
+        <is>
+          <t>Avant Gifting Solutions</t>
+        </is>
+      </c>
+      <c r="D79" s="4" t="inlineStr">
+        <is>
+          <t>Mumbai</t>
+        </is>
+      </c>
+      <c r="E79" s="5" t="inlineStr"/>
+      <c r="F79" s="4" t="inlineStr">
+        <is>
+          <t>Supply handwoven trays, baskets and boxes as bases for their trousseau &amp; gift packing</t>
+        </is>
+      </c>
+      <c r="G79" s="5" t="inlineStr"/>
+      <c r="H79" s="5" t="inlineStr"/>
+      <c r="I79" s="4" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J79" s="5" t="inlineStr"/>
+      <c r="K79" s="5" t="inlineStr"/>
+      <c r="L79" s="4" t="inlineStr">
+        <is>
+          <t>https://www.wedmegood.com/vendors/mumbai/trousseau-packers/</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="4" t="n">
+        <v>79</v>
+      </c>
+      <c r="B80" s="4" t="inlineStr">
+        <is>
+          <t>Trousseau / wedding gift packers</t>
+        </is>
+      </c>
+      <c r="C80" s="4" t="inlineStr">
+        <is>
+          <t>Dottedi</t>
+        </is>
+      </c>
+      <c r="D80" s="4" t="inlineStr">
+        <is>
+          <t>Thane / pan-India</t>
+        </is>
+      </c>
+      <c r="E80" s="5" t="inlineStr"/>
+      <c r="F80" s="4" t="inlineStr">
+        <is>
+          <t>Supply handwoven trays, baskets and boxes as bases for their trousseau &amp; gift packing</t>
+        </is>
+      </c>
+      <c r="G80" s="5" t="inlineStr"/>
+      <c r="H80" s="5" t="inlineStr"/>
+      <c r="I80" s="4" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J80" s="5" t="inlineStr"/>
+      <c r="K80" s="5" t="inlineStr"/>
+      <c r="L80" s="4" t="inlineStr">
+        <is>
+          <t>https://mytribe.in/dotted-i/wedding-gifting-trousseau-packing/featured</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="4" t="n">
+        <v>80</v>
+      </c>
+      <c r="B81" s="4" t="inlineStr">
+        <is>
+          <t>Trousseau / wedding gift packers</t>
+        </is>
+      </c>
+      <c r="C81" s="4" t="inlineStr">
+        <is>
+          <t>Collected Thread</t>
+        </is>
+      </c>
+      <c r="D81" s="4" t="inlineStr">
+        <is>
+          <t>Kolkata (Ballygunge)</t>
+        </is>
+      </c>
+      <c r="E81" s="5" t="inlineStr"/>
+      <c r="F81" s="4" t="inlineStr">
+        <is>
+          <t>Supply handwoven trays, baskets and boxes as bases for their trousseau &amp; gift packing</t>
+        </is>
+      </c>
+      <c r="G81" s="5" t="inlineStr"/>
+      <c r="H81" s="5" t="inlineStr"/>
+      <c r="I81" s="4" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J81" s="5" t="inlineStr"/>
+      <c r="K81" s="5" t="inlineStr"/>
+      <c r="L81" s="4" t="inlineStr">
+        <is>
+          <t>https://www.weddingwire.in/trousseau-packing/kolkata</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="4" t="n">
+        <v>81</v>
+      </c>
+      <c r="B82" s="4" t="inlineStr">
+        <is>
+          <t>Trousseau / wedding gift packers</t>
+        </is>
+      </c>
+      <c r="C82" s="4" t="inlineStr">
+        <is>
+          <t>Melbandhan</t>
+        </is>
+      </c>
+      <c r="D82" s="4" t="inlineStr">
+        <is>
+          <t>Kolkata</t>
+        </is>
+      </c>
+      <c r="E82" s="5" t="inlineStr"/>
+      <c r="F82" s="4" t="inlineStr">
+        <is>
+          <t>Supply handwoven trays, baskets and boxes as bases for their trousseau &amp; gift packing</t>
+        </is>
+      </c>
+      <c r="G82" s="5" t="inlineStr"/>
+      <c r="H82" s="5" t="inlineStr"/>
+      <c r="I82" s="4" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J82" s="5" t="inlineStr"/>
+      <c r="K82" s="5" t="inlineStr"/>
+      <c r="L82" s="4" t="inlineStr">
+        <is>
+          <t>https://www.weddingwire.in/trousseau-packing/kolkata</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="B83" s="4" t="inlineStr">
+        <is>
+          <t>Trousseau / wedding gift packers</t>
+        </is>
+      </c>
+      <c r="C83" s="4" t="inlineStr">
+        <is>
+          <t>The Decor Trunk</t>
+        </is>
+      </c>
+      <c r="D83" s="4" t="inlineStr">
+        <is>
+          <t>Kolkata</t>
+        </is>
+      </c>
+      <c r="E83" s="5" t="inlineStr"/>
+      <c r="F83" s="4" t="inlineStr">
+        <is>
+          <t>Supply handwoven trays, baskets and boxes as bases for their trousseau &amp; gift packing</t>
+        </is>
+      </c>
+      <c r="G83" s="5" t="inlineStr"/>
+      <c r="H83" s="5" t="inlineStr"/>
+      <c r="I83" s="4" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J83" s="5" t="inlineStr"/>
+      <c r="K83" s="5" t="inlineStr"/>
+      <c r="L83" s="4" t="inlineStr">
+        <is>
+          <t>https://www.weddingwire.in/trousseau-packing/kolkata</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="4" t="n">
+        <v>83</v>
+      </c>
+      <c r="B84" s="4" t="inlineStr">
+        <is>
+          <t>Trousseau / wedding gift packers</t>
+        </is>
+      </c>
+      <c r="C84" s="4" t="inlineStr">
+        <is>
+          <t>Anuradha's Tatwas</t>
+        </is>
+      </c>
+      <c r="D84" s="4" t="inlineStr">
+        <is>
+          <t>Kolkata (Kasba)</t>
+        </is>
+      </c>
+      <c r="E84" s="5" t="inlineStr"/>
+      <c r="F84" s="4" t="inlineStr">
+        <is>
+          <t>Supply handwoven trays, baskets and boxes as bases for their trousseau &amp; gift packing</t>
+        </is>
+      </c>
+      <c r="G84" s="5" t="inlineStr"/>
+      <c r="H84" s="5" t="inlineStr"/>
+      <c r="I84" s="4" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J84" s="5" t="inlineStr"/>
+      <c r="K84" s="5" t="inlineStr"/>
+      <c r="L84" s="4" t="inlineStr">
+        <is>
+          <t>https://www.weddingwire.in/trousseau-packing/kolkata</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="4" t="n">
+        <v>84</v>
+      </c>
+      <c r="B85" s="4" t="inlineStr">
+        <is>
+          <t>Trousseau / wedding gift packers</t>
+        </is>
+      </c>
+      <c r="C85" s="4" t="inlineStr">
+        <is>
+          <t>Petal Crafts</t>
+        </is>
+      </c>
+      <c r="D85" s="4" t="inlineStr">
+        <is>
+          <t>Kolkata (Alipore)</t>
+        </is>
+      </c>
+      <c r="E85" s="5" t="inlineStr"/>
+      <c r="F85" s="4" t="inlineStr">
+        <is>
+          <t>Supply handwoven trays, baskets and boxes as bases for their trousseau &amp; gift packing</t>
+        </is>
+      </c>
+      <c r="G85" s="5" t="inlineStr"/>
+      <c r="H85" s="5" t="inlineStr"/>
+      <c r="I85" s="4" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J85" s="5" t="inlineStr"/>
+      <c r="K85" s="5" t="inlineStr"/>
+      <c r="L85" s="4" t="inlineStr">
+        <is>
+          <t>https://www.weddingwire.in/trousseau-packing/kolkata</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="4" t="n">
+        <v>85</v>
+      </c>
+      <c r="B86" s="4" t="inlineStr">
+        <is>
+          <t>Trousseau / wedding gift packers</t>
+        </is>
+      </c>
+      <c r="C86" s="4" t="inlineStr">
+        <is>
+          <t>Purple Tulips</t>
+        </is>
+      </c>
+      <c r="D86" s="4" t="inlineStr">
+        <is>
+          <t>Bengaluru (Horamavu)</t>
+        </is>
+      </c>
+      <c r="E86" s="5" t="inlineStr"/>
+      <c r="F86" s="4" t="inlineStr">
+        <is>
+          <t>Supply handwoven trays, baskets and boxes as bases for their trousseau &amp; gift packing</t>
+        </is>
+      </c>
+      <c r="G86" s="5" t="inlineStr"/>
+      <c r="H86" s="5" t="inlineStr"/>
+      <c r="I86" s="4" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J86" s="5" t="inlineStr"/>
+      <c r="K86" s="5" t="inlineStr"/>
+      <c r="L86" s="4" t="inlineStr">
+        <is>
+          <t>https://www.indiamart.com/purple-tulips/other-services.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="4" t="n">
+        <v>86</v>
+      </c>
+      <c r="B87" s="4" t="inlineStr">
+        <is>
+          <t>Trousseau / wedding gift packers</t>
+        </is>
+      </c>
+      <c r="C87" s="4" t="inlineStr">
+        <is>
+          <t>INAARA</t>
+        </is>
+      </c>
+      <c r="D87" s="4" t="inlineStr">
+        <is>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="E87" s="5" t="inlineStr"/>
+      <c r="F87" s="4" t="inlineStr">
+        <is>
+          <t>Supply handwoven trays, baskets and boxes as bases for their trousseau &amp; gift packing</t>
+        </is>
+      </c>
+      <c r="G87" s="5" t="inlineStr"/>
+      <c r="H87" s="5" t="inlineStr"/>
+      <c r="I87" s="4" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J87" s="5" t="inlineStr"/>
+      <c r="K87" s="5" t="inlineStr"/>
+      <c r="L87" s="4" t="inlineStr">
+        <is>
+          <t>https://www.wedmegood.com/vendors/bangalore/trousseau-packers/</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="4" t="n">
+        <v>87</v>
+      </c>
+      <c r="B88" s="4" t="inlineStr">
+        <is>
+          <t>Trousseau / wedding gift packers</t>
+        </is>
+      </c>
+      <c r="C88" s="4" t="inlineStr">
+        <is>
+          <t>Desi Krafts</t>
+        </is>
+      </c>
+      <c r="D88" s="4" t="inlineStr">
+        <is>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="E88" s="5" t="inlineStr"/>
+      <c r="F88" s="4" t="inlineStr">
+        <is>
+          <t>Supply handwoven trays, baskets and boxes as bases for their trousseau &amp; gift packing</t>
+        </is>
+      </c>
+      <c r="G88" s="5" t="inlineStr"/>
+      <c r="H88" s="5" t="inlineStr"/>
+      <c r="I88" s="4" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J88" s="5" t="inlineStr"/>
+      <c r="K88" s="5" t="inlineStr"/>
+      <c r="L88" s="4" t="inlineStr">
+        <is>
+          <t>https://www.wedmegood.com/vendors/bangalore/trousseau-packers/</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="4" t="n">
+        <v>88</v>
+      </c>
+      <c r="B89" s="4" t="inlineStr">
+        <is>
+          <t>Trousseau / wedding gift packers</t>
+        </is>
+      </c>
+      <c r="C89" s="4" t="inlineStr">
+        <is>
+          <t>RK Giftora</t>
+        </is>
+      </c>
+      <c r="D89" s="4" t="inlineStr">
+        <is>
+          <t>Chandigarh / pan-India</t>
+        </is>
+      </c>
+      <c r="E89" s="5" t="inlineStr"/>
+      <c r="F89" s="4" t="inlineStr">
+        <is>
+          <t>Supply handwoven trays, baskets and boxes as bases for their trousseau &amp; gift packing</t>
+        </is>
+      </c>
+      <c r="G89" s="5" t="inlineStr"/>
+      <c r="H89" s="5" t="inlineStr"/>
+      <c r="I89" s="4" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J89" s="5" t="inlineStr"/>
+      <c r="K89" s="5" t="inlineStr"/>
+      <c r="L89" s="4" t="inlineStr">
+        <is>
+          <t>https://rkgiftora.com/pages/wedding-packaging-chandigarh</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="4" t="n">
+        <v>89</v>
+      </c>
+      <c r="B90" s="4" t="inlineStr">
+        <is>
+          <t>Festive hamper brands</t>
+        </is>
+      </c>
+      <c r="C90" s="4" t="inlineStr">
+        <is>
+          <t>Happilo</t>
+        </is>
+      </c>
+      <c r="D90" s="4" t="inlineStr">
+        <is>
+          <t>Bengaluru</t>
+        </is>
+      </c>
+      <c r="E90" s="5" t="inlineStr"/>
+      <c r="F90" s="4" t="inlineStr">
+        <is>
+          <t>Reusable handwoven baskets/trays to replace plastic or cardboard hamper packaging</t>
+        </is>
+      </c>
+      <c r="G90" s="5" t="inlineStr"/>
+      <c r="H90" s="5" t="inlineStr"/>
+      <c r="I90" s="4" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J90" s="5" t="inlineStr"/>
+      <c r="K90" s="5" t="inlineStr"/>
+      <c r="L90" s="4" t="inlineStr">
+        <is>
+          <t>https://www.flipkart.com/happilo-dry-fruit-celebration-gift-box-robin-ideal-rakhi-corporate-gifts-family-assorted-nuts/p/itm17d351a687605</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="4" t="n">
+        <v>90</v>
+      </c>
+      <c r="B91" s="4" t="inlineStr">
+        <is>
+          <t>Festive hamper brands</t>
+        </is>
+      </c>
+      <c r="C91" s="4" t="inlineStr">
+        <is>
+          <t>Nutraj</t>
+        </is>
+      </c>
+      <c r="D91" s="4" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="E91" s="5" t="inlineStr"/>
+      <c r="F91" s="4" t="inlineStr">
+        <is>
+          <t>Reusable handwoven baskets/trays to replace plastic or cardboard hamper packaging</t>
+        </is>
+      </c>
+      <c r="G91" s="5" t="inlineStr"/>
+      <c r="H91" s="5" t="inlineStr"/>
+      <c r="I91" s="4" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J91" s="5" t="inlineStr"/>
+      <c r="K91" s="5" t="inlineStr"/>
+      <c r="L91" s="4" t="inlineStr">
+        <is>
+          <t>https://www.nutraj.com/collections/gifting</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="4" t="n">
+        <v>91</v>
+      </c>
+      <c r="B92" s="4" t="inlineStr">
+        <is>
+          <t>Festive hamper brands</t>
+        </is>
+      </c>
+      <c r="C92" s="4" t="inlineStr">
+        <is>
+          <t>Farmley</t>
+        </is>
+      </c>
+      <c r="D92" s="4" t="inlineStr">
+        <is>
+          <t>Delhi NCR</t>
+        </is>
+      </c>
+      <c r="E92" s="5" t="inlineStr"/>
+      <c r="F92" s="4" t="inlineStr">
+        <is>
+          <t>Reusable handwoven baskets/trays to replace plastic or cardboard hamper packaging</t>
+        </is>
+      </c>
+      <c r="G92" s="5" t="inlineStr"/>
+      <c r="H92" s="5" t="inlineStr"/>
+      <c r="I92" s="4" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J92" s="5" t="inlineStr"/>
+      <c r="K92" s="5" t="inlineStr"/>
+      <c r="L92" s="4" t="inlineStr">
+        <is>
+          <t>https://www.amazon.in/Dried-Fruits/b?ie=UTF8&amp;node=4859612031</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="4" t="n">
+        <v>92</v>
+      </c>
+      <c r="B93" s="4" t="inlineStr">
+        <is>
+          <t>Festive hamper brands</t>
+        </is>
+      </c>
+      <c r="C93" s="4" t="inlineStr">
+        <is>
+          <t>Chau Foods</t>
+        </is>
+      </c>
+      <c r="D93" s="4" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="E93" s="5" t="inlineStr"/>
+      <c r="F93" s="4" t="inlineStr">
+        <is>
+          <t>Reusable handwoven baskets/trays to replace plastic or cardboard hamper packaging</t>
+        </is>
+      </c>
+      <c r="G93" s="5" t="inlineStr"/>
+      <c r="H93" s="5" t="inlineStr"/>
+      <c r="I93" s="4" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J93" s="5" t="inlineStr"/>
+      <c r="K93" s="5" t="inlineStr"/>
+      <c r="L93" s="4" t="inlineStr">
+        <is>
+          <t>https://www.chaufoods.com/best-dry-fruit-brand-in-india</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="4" t="n">
+        <v>93</v>
+      </c>
+      <c r="B94" s="4" t="inlineStr">
+        <is>
+          <t>Corporates (direct buyers)</t>
+        </is>
+      </c>
+      <c r="C94" s="4" t="inlineStr">
+        <is>
+          <t>HCLTech</t>
+        </is>
+      </c>
+      <c r="D94" s="4" t="inlineStr">
+        <is>
+          <t>Noida</t>
+        </is>
+      </c>
+      <c r="E94" s="5" t="inlineStr"/>
+      <c r="F94" s="4" t="inlineStr">
+        <is>
+          <t>Warm intro via your client My E-haat / HCL Foundation</t>
+        </is>
+      </c>
+      <c r="G94" s="5" t="inlineStr"/>
+      <c r="H94" s="5" t="inlineStr"/>
+      <c r="I94" s="4" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J94" s="5" t="inlineStr"/>
+      <c r="K94" s="5" t="inlineStr"/>
+      <c r="L94" s="4" t="inlineStr">
+        <is>
+          <t>https://indiacsr.in/csr-hcl-foundation-launched-my-e-haat-display-center-in-noida</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="4" t="n">
+        <v>94</v>
+      </c>
+      <c r="B95" s="4" t="inlineStr">
+        <is>
+          <t>Corporates (direct buyers)</t>
+        </is>
+      </c>
+      <c r="C95" s="4" t="inlineStr">
+        <is>
+          <t>Deloitte India</t>
+        </is>
+      </c>
+      <c r="D95" s="4" t="inlineStr">
+        <is>
+          <t>Pan-India</t>
+        </is>
+      </c>
+      <c r="E95" s="5" t="inlineStr"/>
+      <c r="F95" s="4" t="inlineStr">
+        <is>
+          <t>Already buys artisan-made bulk gifts (per Kari by Kriti)</t>
+        </is>
+      </c>
+      <c r="G95" s="5" t="inlineStr"/>
+      <c r="H95" s="5" t="inlineStr"/>
+      <c r="I95" s="4" t="inlineStr">
+        <is>
+          <t>Not contacted</t>
+        </is>
+      </c>
+      <c r="J95" s="5" t="inlineStr"/>
+      <c r="K95" s="5" t="inlineStr"/>
+      <c r="L95" s="4" t="inlineStr">
+        <is>
+          <t>https://www.karibykriti.com/blogs/news/sustainable-corporate-diwali-gifts-india-2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L41"/>
+  <autoFilter ref="A1:L95"/>
   <dataValidations count="1">
-    <dataValidation sqref="I2:I41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I95" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not contacted,Connected,Messaged,Replied,Samples sent,Quote sent,Won,Lost"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2256,7 +4416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2425,6 +4585,33 @@
       <c r="E6" s="4" t="inlineStr">
         <is>
           <t>Hi {name}, swap plastic/cardboard hamper bases for handwoven baskets and trays your customers reuse. We supply in bulk with custom sizes. Interested in samples for Diwali?</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Trousseau / wedding gift packers</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Founder OR Owner</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>trousseau packing OR gift packing OR hampers</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Delhi, Mumbai, Kolkata, Bengaluru, Chandigarh</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Hi {name}, we make handwoven grass trays, baskets and boxes that make trousseau packing look premium and plastic-free. Bulk rates for packers – could I send a sample set?</t>
         </is>
       </c>
     </row>

</xml_diff>